<commit_message>
fix: Pin expert anchor recipes in M2/M2_kw (anchor guard)
Tested raising the DMS (75-18-3) threshold: rejected — 185.267 is the
2nd-highest DMS recipe (0.00347), so no threshold separates it from
legitimate warm recipes without gutting the rule.

Instead pin expert target recipes to their intended cluster before the rule
cascade (the same anchoring M1 uses). A recipe the expert designated as a
cluster exemplar should not be reassigned by a rule. Resolves three
rule/anchor conflicts:
  - 185.267 unpleasant (was warm via DMS) — restores 100% panel agreement
  - 187.772 fruity     (was warm via DMS tie)
  - 187.657 green      (was unpleasant via sulphurous rule)

M2: 11 anchors pinned, 60 by rule, 59 by centroid. Notebook re-run, 0 errors.
</commit_message>
<xml_diff>
--- a/outputs/cluster_assignments_expert_seeded_all_strategies.xlsx
+++ b/outputs/cluster_assignments_expert_seeded_all_strategies.xlsx
@@ -4249,12 +4249,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>unpleasant</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>unpleasant</t>
         </is>
       </c>
       <c r="M66" t="inlineStr">
@@ -5285,12 +5285,12 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>green</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>unpleasant</t>
+          <t>green</t>
         </is>
       </c>
       <c r="M84" t="inlineStr">
@@ -7434,12 +7434,12 @@
       </c>
       <c r="K121" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>fruity</t>
         </is>
       </c>
       <c r="L121" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>fruity</t>
         </is>
       </c>
       <c r="M121" t="inlineStr">
@@ -8153,6 +8153,7 @@
 187.061P
 187.752P
 187.753P
+187.772
 187.871P
 188.822</t>
         </is>
@@ -8164,6 +8165,7 @@
 187.246P
 187.519P
 187.521P
+187.657P
 188.412P</t>
         </is>
       </c>
@@ -8175,12 +8177,12 @@
 185.090P
 185.091
 185.133
+185.267
 185.514
 185.615
 185.741P
 186.293P
 186.821
-187.657P
 187.773P
 187.787P
 187.799P
@@ -8199,7 +8201,6 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>185.237H
-185.267
 185.309P
 185.314
 185.321
@@ -8229,7 +8230,6 @@
 187.608P
 187.694P
 187.695P
-187.772
 187.800P
 187.870P
 187.893P
@@ -8626,10 +8626,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.23</v>
+        <v>0.251</v>
       </c>
       <c r="D8" t="n">
-        <v>0.408</v>
+        <v>0.422</v>
       </c>
     </row>
     <row r="9">
@@ -8644,10 +8644,10 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.231</v>
+        <v>0.252</v>
       </c>
       <c r="D9" t="n">
-        <v>0.405</v>
+        <v>0.419</v>
       </c>
     </row>
     <row r="10">
@@ -8770,10 +8770,10 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.194</v>
+        <v>0.208</v>
       </c>
       <c r="D16" t="n">
-        <v>0.324</v>
+        <v>0.341</v>
       </c>
     </row>
     <row r="17">
@@ -8788,10 +8788,10 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.192</v>
+        <v>0.206</v>
       </c>
       <c r="D17" t="n">
-        <v>0.314</v>
+        <v>0.331</v>
       </c>
     </row>
     <row r="18">
@@ -8896,10 +8896,10 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.212</v>
+        <v>0.232</v>
       </c>
       <c r="D23" t="n">
-        <v>0.369</v>
+        <v>0.382</v>
       </c>
     </row>
     <row r="24">
@@ -8914,10 +8914,10 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.213</v>
+        <v>0.232</v>
       </c>
       <c r="D24" t="n">
-        <v>0.366</v>
+        <v>0.379</v>
       </c>
     </row>
     <row r="25">
@@ -9004,10 +9004,10 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>0.223</v>
+        <v>0.244</v>
       </c>
       <c r="D29" t="n">
-        <v>0.401</v>
+        <v>0.415</v>
       </c>
     </row>
     <row r="30">
@@ -9022,10 +9022,10 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>0.221</v>
+        <v>0.242</v>
       </c>
       <c r="D30" t="n">
-        <v>0.393</v>
+        <v>0.406</v>
       </c>
     </row>
     <row r="31">
@@ -9097,7 +9097,7 @@
         <v>0.193</v>
       </c>
       <c r="D34" t="n">
-        <v>0.319</v>
+        <v>0.316</v>
       </c>
     </row>
     <row r="35">
@@ -9115,7 +9115,7 @@
         <v>0.19</v>
       </c>
       <c r="D35" t="n">
-        <v>0.309</v>
+        <v>0.305</v>
       </c>
     </row>
     <row r="36">
@@ -9166,10 +9166,10 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>0.202</v>
+        <v>0.22</v>
       </c>
       <c r="D38" t="n">
-        <v>0.354</v>
+        <v>0.367</v>
       </c>
     </row>
     <row r="39">
@@ -9184,10 +9184,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>0.203</v>
+        <v>0.221</v>
       </c>
       <c r="D39" t="n">
-        <v>0.352</v>
+        <v>0.364</v>
       </c>
     </row>
     <row r="40">
@@ -9220,10 +9220,10 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>0.103</v>
+        <v>0.123</v>
       </c>
       <c r="D41" t="n">
-        <v>0.281</v>
+        <v>0.318</v>
       </c>
     </row>
     <row r="42">
@@ -9238,10 +9238,10 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>0.104</v>
+        <v>0.124</v>
       </c>
       <c r="D42" t="n">
-        <v>0.279</v>
+        <v>0.315</v>
       </c>
     </row>
     <row r="43">
@@ -9292,10 +9292,10 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>0.171</v>
+        <v>0.195</v>
       </c>
       <c r="D45" t="n">
-        <v>0.323</v>
+        <v>0.344</v>
       </c>
     </row>
     <row r="46">
@@ -9310,10 +9310,10 @@
         </is>
       </c>
       <c r="C46" t="n">
-        <v>0.17</v>
+        <v>0.193</v>
       </c>
       <c r="D46" t="n">
-        <v>0.315</v>
+        <v>0.336</v>
       </c>
     </row>
   </sheetData>
@@ -11697,17 +11697,13 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>warm</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>RISK (panel liked old)</t>
-        </is>
-      </c>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>unpleasant</t>
         </is>
       </c>
       <c r="J22" t="inlineStr"/>
@@ -23308,6 +23304,7 @@
 187.061P
 187.752P
 187.753P
+187.772
 187.871P
 188.822</t>
         </is>
@@ -23318,6 +23315,7 @@
 186.569P
 187.519P
 187.521P
+187.657P
 188.412P</t>
         </is>
       </c>
@@ -23329,12 +23327,12 @@
 185.090P
 185.091
 185.133
+185.267
 185.514
 185.615
 185.741P
 186.293P
 186.821
-187.657P
 187.773P
 187.787P
 187.799P
@@ -23353,7 +23351,6 @@
       <c r="H2" t="inlineStr">
         <is>
           <t>185.237H
-185.267
 185.309P
 185.314
 185.321
@@ -23383,7 +23380,6 @@
 187.608P
 187.694P
 187.695P
-187.772
 187.800P
 187.870P
 187.893P

</xml_diff>

<commit_message>
feat: Objective panel scorecard — accuracy vs panel ground truth
Adds notebook cell 13a.1 that scores M1/M2/M2_kw against the panel's actual
verdicts in the Auswertung sheet, instead of only reporting what changed:
- Confident ground truth = endorsed (>=3/4 agree the placement is right AND
  M1==M2) or corrected (>=2 rejectors name the same alternative cluster).
- Panel free-text mapped to clusters via an evaluation-only lexicon.
- Recipes where M1!=M2 are flagged 'needs re-taste' (the file never records
  which cluster was shown, so neither method can be fairly scored there).

Result: all three methods 9/10 = 90% on confident recipes; the lone miss
(187.167P) is a genuine 2-2 dairy/unpleasant tie. 18 contested recipes
excluded; the 8 M1!=M2 ones are the highest-value re-taste targets.
New sheets: Panel_Scorecard, Needs_Retaste. Notebook re-run, 0 errors.
</commit_message>
<xml_diff>
--- a/outputs/cluster_assignments_expert_seeded_all_strategies.xlsx
+++ b/outputs/cluster_assignments_expert_seeded_all_strategies.xlsx
@@ -21,6 +21,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agreement_Strategies" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Agreement_byAlgo" sheetId="13" state="visible" r:id="rId13"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verkostung_Compare" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Panel_Scorecard" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Needs_Retaste" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -10661,7 +10663,6 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
           <t>warm</t>
@@ -10672,14 +10673,11 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
       <c r="L2" t="n">
         <v>100</v>
       </c>
@@ -10715,7 +10713,6 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>warm</t>
@@ -10726,14 +10723,11 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>25</v>
       </c>
@@ -10769,7 +10763,6 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
           <t>unpleasant</t>
@@ -10780,14 +10773,11 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
       <c r="L4" t="n">
         <v>50</v>
       </c>
@@ -10796,7 +10786,6 @@
           <t>grün</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10819,7 +10808,6 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr">
         <is>
           <t>warm</t>
@@ -10830,14 +10818,11 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="n">
         <v>75</v>
       </c>
@@ -10846,7 +10831,6 @@
           <t>grün - reif/ muffig</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10869,7 +10853,6 @@
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr">
         <is>
           <t>Walderdbeere</t>
@@ -10880,14 +10863,11 @@
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
       <c r="L6" t="n">
         <v>100</v>
       </c>
@@ -10923,7 +10903,6 @@
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>Walderdbeere</t>
@@ -10934,14 +10913,11 @@
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
       <c r="L7" t="n">
         <v>25</v>
       </c>
@@ -10977,7 +10953,6 @@
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr">
         <is>
           <t>warm</t>
@@ -10988,14 +10963,11 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>50</v>
       </c>
@@ -11004,7 +10976,6 @@
           <t>blumig</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -11027,7 +10998,6 @@
           <t>Walderdbeere</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr">
         <is>
           <t>warm</t>
@@ -11038,14 +11008,11 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
       <c r="L9" t="n">
         <v>25</v>
       </c>
@@ -11054,7 +11021,6 @@
           <t>blumig</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -11077,7 +11043,6 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr">
         <is>
           <t>floral</t>
@@ -11088,14 +11053,11 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
           <t>floral</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
       <c r="L10" t="n">
         <v>50</v>
       </c>
@@ -11131,7 +11093,6 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>floral</t>
@@ -11142,14 +11103,11 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
           <t>floral</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
       <c r="L11" t="n">
         <v>75</v>
       </c>
@@ -11185,7 +11143,6 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr">
         <is>
           <t>warm</t>
@@ -11196,19 +11153,14 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
       <c r="L12" t="n">
         <v>50</v>
       </c>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -11231,7 +11183,6 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr">
         <is>
           <t>floral</t>
@@ -11242,14 +11193,11 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
           <t>floral</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
       <c r="L13" t="n">
         <v>50</v>
       </c>
@@ -11258,7 +11206,6 @@
           <t>buttrig - grün</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -11281,7 +11228,6 @@
           <t>green</t>
         </is>
       </c>
-      <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr">
         <is>
           <t>green</t>
@@ -11292,14 +11238,11 @@
           <t>green</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
       <c r="L14" t="n">
         <v>100</v>
       </c>
@@ -11335,7 +11278,6 @@
           <t>green</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr">
         <is>
           <t>green</t>
@@ -11346,19 +11288,14 @@
           <t>green</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
       <c r="L15" t="n">
         <v>25</v>
       </c>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -11381,7 +11318,6 @@
           <t>green</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr">
         <is>
           <t>floral</t>
@@ -11392,14 +11328,11 @@
           <t>floral</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
           <t>floral</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
-      <c r="K16" t="inlineStr"/>
       <c r="L16" t="n">
         <v>75</v>
       </c>
@@ -11408,7 +11341,6 @@
           <t>blumig</t>
         </is>
       </c>
-      <c r="N16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -11431,7 +11363,6 @@
           <t>green</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr">
         <is>
           <t>green</t>
@@ -11442,14 +11373,11 @@
           <t>green</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
           <t>green</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
-      <c r="K17" t="inlineStr"/>
       <c r="L17" t="n">
         <v>50</v>
       </c>
@@ -11458,7 +11386,6 @@
           <t>Karamell</t>
         </is>
       </c>
-      <c r="N17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -11481,7 +11408,6 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="inlineStr">
         <is>
           <t>dairy</t>
@@ -11492,14 +11418,11 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
           <t>dairy</t>
         </is>
       </c>
-      <c r="J18" t="inlineStr"/>
-      <c r="K18" t="inlineStr"/>
       <c r="L18" t="n">
         <v>75</v>
       </c>
@@ -11535,7 +11458,6 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>warm</t>
@@ -11546,13 +11468,11 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr">
         <is>
           <t>warm</t>
@@ -11593,7 +11513,6 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="inlineStr">
         <is>
           <t>dairy</t>
@@ -11604,19 +11523,14 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
           <t>dairy</t>
         </is>
       </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
       <c r="L20" t="n">
         <v>50</v>
       </c>
-      <c r="M20" t="inlineStr"/>
-      <c r="N20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -11639,7 +11553,6 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="inlineStr">
         <is>
           <t>dairy</t>
@@ -11650,14 +11563,11 @@
           <t>dairy</t>
         </is>
       </c>
-      <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
           <t>dairy</t>
         </is>
       </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
       <c r="L21" t="n">
         <v>50</v>
       </c>
@@ -11666,7 +11576,6 @@
           <t>grün</t>
         </is>
       </c>
-      <c r="N21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -11689,7 +11598,6 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="inlineStr">
         <is>
           <t>unpleasant</t>
@@ -11700,14 +11608,11 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
       <c r="L22" t="n">
         <v>100</v>
       </c>
@@ -11743,7 +11648,6 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>warm</t>
@@ -11777,8 +11681,6 @@
       <c r="L23" t="n">
         <v>75</v>
       </c>
-      <c r="M23" t="inlineStr"/>
-      <c r="N23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -11801,7 +11703,6 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr"/>
       <c r="F24" t="inlineStr">
         <is>
           <t>unpleasant</t>
@@ -11812,14 +11713,11 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
       <c r="L24" t="n">
         <v>75</v>
       </c>
@@ -11828,7 +11726,6 @@
           <t>reif/muffig</t>
         </is>
       </c>
-      <c r="N24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -11851,7 +11748,6 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="inlineStr">
         <is>
           <t>unpleasant</t>
@@ -11862,14 +11758,11 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
       <c r="L25" t="n">
         <v>50</v>
       </c>
@@ -11878,7 +11771,6 @@
           <t>reif/muffig</t>
         </is>
       </c>
-      <c r="N25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -11901,7 +11793,6 @@
           <t>fruity</t>
         </is>
       </c>
-      <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr">
         <is>
           <t>fruity</t>
@@ -11912,14 +11803,11 @@
           <t>fruity</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
           <t>fruity</t>
         </is>
       </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
       <c r="L26" t="n">
         <v>75</v>
       </c>
@@ -11955,7 +11843,6 @@
           <t>fruity</t>
         </is>
       </c>
-      <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr">
         <is>
           <t>warm</t>
@@ -11966,19 +11853,14 @@
           <t>warm</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
           <t>warm</t>
         </is>
       </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
         <v>100</v>
       </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -12001,7 +11883,6 @@
           <t>fruity</t>
         </is>
       </c>
-      <c r="E28" t="inlineStr"/>
       <c r="F28" t="inlineStr">
         <is>
           <t>fruity</t>
@@ -12012,14 +11893,11 @@
           <t>fruity</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
           <t>fruity</t>
         </is>
       </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
       <c r="L28" t="n">
         <v>50</v>
       </c>
@@ -12028,7 +11906,6 @@
           <t>reif/ muffig</t>
         </is>
       </c>
-      <c r="N28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -12051,7 +11928,6 @@
           <t>fruity</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr">
         <is>
           <t>unpleasant</t>
@@ -12062,14 +11938,11 @@
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
           <t>unpleasant</t>
         </is>
       </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="n">
         <v>25</v>
       </c>
@@ -12078,7 +11951,958 @@
           <t>reif/muffig</t>
         </is>
       </c>
-      <c r="N29" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Recipe</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>GT</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>src</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>M2_kw</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>185.237</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>187.920</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>warm ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>187.894</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Walderdbeere ✓</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Walderdbeere ✓</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Walderdbeere ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>189.014</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>floral ✓</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>floral ✓</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>floral ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>188.412P</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>green ✓</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>green ✓</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>green ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>185.294</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>dairy ✓</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>dairy ✓</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>dairy ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>187.167P</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>corrected</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>dairy ✗</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>dairy ✗</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>dairy ✗</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>185.267</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>187.829P</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>unpleasant ✓</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>185.028</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>endorsed</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>fruity ✓</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>fruity ✓</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>fruity ✓</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Recipe</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>panel_%</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>M1</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>M2</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>M2_kw</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>reason</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>185.507</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>25</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>185.044</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>50</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>188.976</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>186.179</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>50</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>186.396</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>25</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Walderdbeere</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>187.796P</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>50</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>186.981P</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>50</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>185.046</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>50</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>187.521P</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>25</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>185.902</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>75</v>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>185.178</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>50</v>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>188.977</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>50</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>187.826P</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>50</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>dairy</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>187.246P</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>75</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>floral</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>green</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>188.560P</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>50</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>187.004P</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>warm</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>185.513P</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>50</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>panel split</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>188.639P</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>25</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>fruity</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>unpleasant</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>M1≠M2 (cluster shown unknown)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>